<commit_message>
update 2014 and 2017 local election, regenerate registries
</commit_message>
<xml_diff>
--- a/src/data/raw/2014 შუალედური.xlsx
+++ b/src/data/raw/2014 შუალედური.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Election portal data sets\Election results\შედეგები\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\My projects\Elections\ge_elections_dashboard\wireframe\observable_framework\elections_data\src\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A9988F-D466-4BBC-A11D-096E6017F7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA8CC50-CDE2-4062-9675-3B3860ED3A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1491" yWindow="540" windowWidth="28775" windowHeight="17254" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="48.05 ვახანი" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>ოლქის N და დასახელება</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>41 მერაბ ღონღაძე</t>
+  </si>
+  <si>
+    <t>maj_id</t>
   </si>
 </sst>
 </file>
@@ -443,145 +446,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="15.07421875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.69140625" customWidth="1"/>
-    <col min="3" max="3" width="10.4609375" customWidth="1"/>
-    <col min="4" max="4" width="20.07421875" customWidth="1"/>
-    <col min="5" max="5" width="19.69140625" customWidth="1"/>
-    <col min="6" max="6" width="12.53515625" customWidth="1"/>
-    <col min="7" max="7" width="12.84375" customWidth="1"/>
-    <col min="8" max="8" width="15.53515625" customWidth="1"/>
-    <col min="9" max="9" width="18.07421875" customWidth="1"/>
-    <col min="10" max="11" width="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="15.07421875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.69140625" customWidth="1"/>
+    <col min="4" max="4" width="10.4609375" customWidth="1"/>
+    <col min="5" max="5" width="20.07421875" customWidth="1"/>
+    <col min="6" max="6" width="19.69140625" customWidth="1"/>
+    <col min="7" max="7" width="12.53515625" customWidth="1"/>
+    <col min="8" max="8" width="12.84375" customWidth="1"/>
+    <col min="9" max="9" width="15.53515625" customWidth="1"/>
+    <col min="10" max="10" width="18.07421875" customWidth="1"/>
+    <col min="11" max="12" width="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.3046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="102.45" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="102.45" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
+        <v>4805</v>
+      </c>
+      <c r="B2" s="1">
         <v>48</v>
       </c>
-      <c r="B2" s="1">
+      <c r="C2" s="1">
         <v>5</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2" s="1">
         <v>9</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>732</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>0</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>78</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>202</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>265</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>700</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="1">
         <v>62</v>
       </c>
-      <c r="K2" s="1">
+      <c r="L2" s="1">
         <v>195</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="5"/>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="C3" s="5"/>
-      <c r="D3" s="5">
-        <f>D2</f>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5">
+        <f>E2</f>
         <v>732</v>
       </c>
-      <c r="E3" s="5">
-        <f t="shared" ref="E3:L3" si="0">E2</f>
+      <c r="F3" s="5">
+        <f t="shared" ref="F3:M3" si="0">F2</f>
         <v>0</v>
       </c>
-      <c r="F3" s="5">
+      <c r="G3" s="5">
         <f t="shared" si="0"/>
         <v>78</v>
       </c>
-      <c r="G3" s="5">
+      <c r="H3" s="5">
         <f t="shared" si="0"/>
         <v>202</v>
       </c>
-      <c r="H3" s="5">
+      <c r="I3" s="5">
         <f t="shared" si="0"/>
         <v>265</v>
       </c>
-      <c r="I3" s="5">
+      <c r="J3" s="5">
         <f t="shared" si="0"/>
         <v>700</v>
       </c>
-      <c r="J3" s="5">
+      <c r="K3" s="5">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="K3" s="5">
+      <c r="L3" s="5">
         <f t="shared" si="0"/>
         <v>195</v>
       </c>
-      <c r="L3" s="5">
+      <c r="M3" s="5">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:L3">
+  <conditionalFormatting sqref="A2:M3">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$C2="ჯამი"</formula>
+      <formula>$D2="ჯამი"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.17" right="0.17" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>